<commit_message>
Add revised research figures and data
This commit adds the revised R scripts, source CSV data, generated figure PNGs, and session metadata for the FREL analyses. It updates the figure-generation code to use the Okabe-Ito palette and reproducible plotting logic for Figures 1-4, and records the final results workbook and environment details.
</commit_message>
<xml_diff>
--- a/results/results_vfinal.xlsx
+++ b/results/results_vfinal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ipamamazonia-my.sharepoint.com/personal/celso_junior_ipam_org_br/Documents/Documentos/GitHub/Brazil-National-FREL/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/celsojunior/Documents/GitHub/Brazil-National-FREL/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{BF2C95EF-3402-44DC-AD55-6CFF0EAF20AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{749A3931-4591-4CA2-A0D8-5F37CED72160}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B36B80CB-3CD0-5149-9BDE-6A955437DA49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-105" windowWidth="38640" windowHeight="15720" tabRatio="761" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="200" yWindow="680" windowWidth="18500" windowHeight="17820" tabRatio="761" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure 1" sheetId="11" r:id="rId1"/>
@@ -665,6 +665,12 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFD55E00"/>
+      <color rgb="FF56B4E9"/>
+      <color rgb="FF0072B2"/>
+      <color rgb="FF1A1A1A"/>
+      <color rgb="FF333333"/>
+      <color rgb="FFE69F00"/>
       <color rgb="FFDE6C6A"/>
       <color rgb="FFE8C75A"/>
       <color rgb="FFF5F4EB"/>
@@ -718,9 +724,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="DE6C6A">
-                <a:alpha val="50196"/>
-              </a:srgbClr>
+              <a:srgbClr val="E69F00"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -738,18 +742,13 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="85000"/>
-                        <a:lumOff val="15000"/>
-                      </a:schemeClr>
+                      <a:srgbClr val="1A1A1A"/>
                     </a:solidFill>
                     <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
                     <a:ea typeface="+mn-ea"/>
@@ -853,7 +852,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="DE6C6A"/>
+              <a:srgbClr val="0072B2"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -871,18 +870,13 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="85000"/>
-                        <a:lumOff val="15000"/>
-                      </a:schemeClr>
+                      <a:schemeClr val="bg1"/>
                     </a:solidFill>
                     <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
                     <a:ea typeface="+mn-ea"/>
@@ -1136,18 +1130,13 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="85000"/>
-                        <a:lumOff val="15000"/>
-                      </a:schemeClr>
+                      <a:srgbClr val="333333"/>
                     </a:solidFill>
                     <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
                     <a:ea typeface="+mn-ea"/>
@@ -1295,10 +1284,7 @@
             <a:pPr>
               <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="85000"/>
-                    <a:lumOff val="15000"/>
-                  </a:schemeClr>
+                  <a:srgbClr val="333333"/>
                 </a:solidFill>
                 <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
                 <a:ea typeface="+mn-ea"/>
@@ -1333,10 +1319,7 @@
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="85000"/>
-                        <a:lumOff val="15000"/>
-                      </a:schemeClr>
+                      <a:srgbClr val="333333"/>
                     </a:solidFill>
                     <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
                     <a:ea typeface="+mn-ea"/>
@@ -1344,22 +1327,9 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="pt-BR" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
-                  <a:t>tons</a:t>
+                  <a:rPr lang="pt-BR"/>
+                  <a:t>tons CO2 eq</a:t>
                 </a:r>
-                <a:r>
-                  <a:rPr lang="pt-BR" baseline="0"/>
-                  <a:t> CO</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="pt-BR" baseline="-25000"/>
-                  <a:t>2</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="pt-BR" baseline="0"/>
-                  <a:t> eq</a:t>
-                </a:r>
-                <a:endParaRPr lang="pt-BR"/>
               </a:p>
             </c:rich>
           </c:tx>
@@ -1378,10 +1348,7 @@
               <a:pPr>
                 <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="85000"/>
-                      <a:lumOff val="15000"/>
-                    </a:schemeClr>
+                    <a:srgbClr val="333333"/>
                   </a:solidFill>
                   <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
                   <a:ea typeface="+mn-ea"/>
@@ -1415,10 +1382,7 @@
             <a:pPr>
               <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="85000"/>
-                    <a:lumOff val="15000"/>
-                  </a:schemeClr>
+                  <a:srgbClr val="333333"/>
                 </a:solidFill>
                 <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
                 <a:ea typeface="+mn-ea"/>
@@ -1442,10 +1406,7 @@
                   <a:pPr>
                     <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="85000"/>
-                          <a:lumOff val="15000"/>
-                        </a:schemeClr>
+                        <a:srgbClr val="333333"/>
                       </a:solidFill>
                       <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
                       <a:ea typeface="+mn-ea"/>
@@ -1453,9 +1414,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:rPr lang="pt-BR" b="0" i="0">
-                      <a:effectLst/>
-                    </a:rPr>
+                    <a:rPr lang="pt-BR"/>
                     <a:t>Millions</a:t>
                   </a:r>
                 </a:p>
@@ -1475,10 +1434,7 @@
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="85000"/>
-                        <a:lumOff val="15000"/>
-                      </a:schemeClr>
+                      <a:srgbClr val="333333"/>
                     </a:solidFill>
                     <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
                     <a:ea typeface="+mn-ea"/>
@@ -1516,10 +1472,7 @@
           <a:pPr>
             <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="85000"/>
-                  <a:lumOff val="15000"/>
-                </a:schemeClr>
+                <a:srgbClr val="333333"/>
               </a:solidFill>
               <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
               <a:ea typeface="+mn-ea"/>
@@ -1558,10 +1511,7 @@
       <a:pPr>
         <a:defRPr sz="1200">
           <a:solidFill>
-            <a:schemeClr val="tx1">
-              <a:lumMod val="85000"/>
-              <a:lumOff val="15000"/>
-            </a:schemeClr>
+            <a:srgbClr val="333333"/>
           </a:solidFill>
           <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
         </a:defRPr>
@@ -1614,7 +1564,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="E8C75A"/>
+              <a:srgbClr val="0072B2"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1639,10 +1589,7 @@
                 <a:pPr>
                   <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="85000"/>
-                        <a:lumOff val="15000"/>
-                      </a:schemeClr>
+                      <a:schemeClr val="bg1"/>
                     </a:solidFill>
                     <a:latin typeface="Montserrat" pitchFamily="2" charset="0"/>
                     <a:ea typeface="+mn-ea"/>
@@ -1761,9 +1708,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="E8C75A">
-                <a:alpha val="50196"/>
-              </a:srgbClr>
+              <a:srgbClr val="56B4E9"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -2351,7 +2296,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:srgbClr val="DE6C6A"/>
+                <a:srgbClr val="D55E00"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
               <a:round/>
@@ -2363,11 +2308,11 @@
             <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
-                <a:srgbClr val="DE6C6A"/>
+                <a:srgbClr val="D55E00"/>
               </a:solidFill>
               <a:ln w="28575">
                 <a:solidFill>
-                  <a:srgbClr val="DE6C6A"/>
+                  <a:srgbClr val="D55E00"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -4195,18 +4140,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{746E9525-7C4D-42FA-A23D-D0CEA7AFCD11}">
   <dimension ref="A1:L26"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.109375" customWidth="1"/>
-    <col min="2" max="2" width="4.109375" customWidth="1"/>
+    <col min="1" max="1" width="10.1640625" customWidth="1"/>
+    <col min="2" max="2" width="4.1640625" customWidth="1"/>
     <col min="3" max="3" width="23.33203125" customWidth="1"/>
-    <col min="4" max="4" width="24.44140625" customWidth="1"/>
+    <col min="4" max="4" width="24.5" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="6" width="32.109375" customWidth="1"/>
+    <col min="6" max="6" width="32.1640625" customWidth="1"/>
     <col min="7" max="7" width="31.33203125" customWidth="1"/>
-    <col min="8" max="8" width="29.44140625" customWidth="1"/>
+    <col min="8" max="8" width="29.5" customWidth="1"/>
     <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.109375" customWidth="1"/>
+    <col min="11" max="11" width="19.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="48.75" customHeight="1">
@@ -4443,18 +4388,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A3ACF42-74B5-4EF7-B6B3-6008AC5E4E20}">
   <dimension ref="A1:O41"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="36.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.44140625" customWidth="1"/>
-    <col min="4" max="4" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.5546875" customWidth="1"/>
+    <col min="3" max="3" width="39.5" customWidth="1"/>
+    <col min="4" max="4" width="28.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.5" customWidth="1"/>
     <col min="6" max="6" width="32.33203125" customWidth="1"/>
-    <col min="7" max="7" width="30.44140625" customWidth="1"/>
+    <col min="7" max="7" width="30.5" customWidth="1"/>
     <col min="8" max="8" width="10.6640625" customWidth="1"/>
-    <col min="9" max="9" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.5546875" customWidth="1"/>
-    <col min="13" max="13" width="13.109375" customWidth="1"/>
+    <col min="9" max="9" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5" customWidth="1"/>
+    <col min="13" max="13" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -4773,21 +4718,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DDE237F-5805-4F40-85AC-796F9BE5D6ED}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.109375" customWidth="1"/>
-    <col min="2" max="2" width="21.44140625" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" customWidth="1"/>
+    <col min="1" max="1" width="8.1640625" customWidth="1"/>
+    <col min="2" max="2" width="73" customWidth="1"/>
+    <col min="8" max="8" width="10.5" customWidth="1"/>
     <col min="10" max="10" width="8.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="49.5" customHeight="1">
+    <row r="1" spans="1:9" ht="27" customHeight="1">
       <c r="A1" s="34" t="s">
         <v>14</v>
       </c>
       <c r="B1" s="35"/>
     </row>
-    <row r="2" spans="1:9" ht="16.2">
+    <row r="2" spans="1:9" ht="17">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -4895,12 +4840,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCF00FE4-336D-4E92-B05B-E6E1C4CE89EE}">
   <dimension ref="A1:M19"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.109375" customWidth="1"/>
-    <col min="2" max="2" width="21.44140625" customWidth="1"/>
-    <col min="3" max="3" width="21.109375" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" customWidth="1"/>
+    <col min="1" max="1" width="8.1640625" customWidth="1"/>
+    <col min="2" max="2" width="21.5" customWidth="1"/>
+    <col min="3" max="3" width="21.1640625" customWidth="1"/>
+    <col min="8" max="8" width="10.5" customWidth="1"/>
     <col min="10" max="10" width="8.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4911,7 +4856,7 @@
       </c>
       <c r="C1" s="38"/>
     </row>
-    <row r="2" spans="1:13" ht="16.2">
+    <row r="2" spans="1:13" ht="17">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -5087,14 +5032,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B8347AE-1F9E-406B-BBBE-0167BC334EA0}">
   <dimension ref="A1:J31"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.33203125" customWidth="1"/>
-    <col min="2" max="2" width="18.88671875" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.2">
+    <row r="1" spans="1:10" ht="18">
       <c r="A1" s="14" t="s">
         <v>20</v>
       </c>
@@ -5328,17 +5273,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62090D6-4474-48C5-9F40-1D3B54A5A11B}">
   <dimension ref="A1:L20"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.109375" customWidth="1"/>
+    <col min="7" max="7" width="21.1640625" customWidth="1"/>
     <col min="8" max="8" width="21.33203125" customWidth="1"/>
     <col min="9" max="9" width="23.6640625" customWidth="1"/>
-    <col min="10" max="10" width="23.88671875" customWidth="1"/>
+    <col min="10" max="10" width="23.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="33.75" customHeight="1">

</xml_diff>